<commit_message>
Updating to include LD50 std dev data
</commit_message>
<xml_diff>
--- a/moboCPA/rawdata/CPA cocktails short summary.xlsx
+++ b/moboCPA/rawdata/CPA cocktails short summary.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10114"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10402"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/danemerson/Documents/CMU/01_Research/Projects/CPA/Data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/danemerson/Documents/CMU/01_Research/Projects/CPA/Bayesian Optimization/cpa-bayesian-opt/moboCPA/rawdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4980D362-55B7-2046-82E4-B82E6F4FDE32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BC450FF-C41C-2D41-A044-59944B824310}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="80" yWindow="760" windowWidth="45340" windowHeight="25680" activeTab="1" xr2:uid="{23C5F3F8-64C3-7842-A25B-DE40D5CC2516}"/>
+    <workbookView xWindow="80" yWindow="760" windowWidth="45340" windowHeight="25680" activeTab="2" xr2:uid="{23C5F3F8-64C3-7842-A25B-DE40D5CC2516}"/>
   </bookViews>
   <sheets>
     <sheet name="Individual CPAs" sheetId="3" r:id="rId1"/>
     <sheet name="Cocktails" sheetId="13" r:id="rId2"/>
+    <sheet name="LD50" sheetId="14" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="20">
   <si>
     <t>CPA</t>
   </si>
@@ -91,6 +92,12 @@
   </si>
   <si>
     <t>% viability</t>
+  </si>
+  <si>
+    <t>Standard Deviation</t>
+  </si>
+  <si>
+    <t>% Viability</t>
   </si>
 </sst>
 </file>
@@ -198,7 +205,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -224,14 +231,15 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2787,9 +2795,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -2827,7 +2835,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -2933,7 +2941,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -3075,7 +3083,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -3099,14 +3107,14 @@
       <c r="B2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="16" t="s">
-        <v>2</v>
-      </c>
-      <c r="D2" s="16"/>
-      <c r="E2" s="16"/>
-      <c r="F2" s="16"/>
-      <c r="G2" s="16"/>
-      <c r="H2" s="16"/>
+      <c r="C2" s="17" t="s">
+        <v>2</v>
+      </c>
+      <c r="D2" s="17"/>
+      <c r="E2" s="17"/>
+      <c r="F2" s="17"/>
+      <c r="G2" s="17"/>
+      <c r="H2" s="17"/>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3" s="3"/>
@@ -3139,7 +3147,7 @@
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A4" s="17" t="s">
+      <c r="A4" s="16" t="s">
         <v>6</v>
       </c>
       <c r="B4" s="5">
@@ -3173,7 +3181,7 @@
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A5" s="17"/>
+      <c r="A5" s="16"/>
       <c r="B5" s="5">
         <v>1</v>
       </c>
@@ -3205,7 +3213,7 @@
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A6" s="17"/>
+      <c r="A6" s="16"/>
       <c r="B6" s="5">
         <v>1.5</v>
       </c>
@@ -3237,7 +3245,7 @@
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A7" s="17"/>
+      <c r="A7" s="16"/>
       <c r="B7" s="5">
         <v>2</v>
       </c>
@@ -3269,7 +3277,7 @@
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A8" s="17"/>
+      <c r="A8" s="16"/>
       <c r="B8" s="5">
         <v>2.5</v>
       </c>
@@ -3301,7 +3309,7 @@
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A9" s="17"/>
+      <c r="A9" s="16"/>
       <c r="B9" s="5">
         <v>3</v>
       </c>
@@ -3333,7 +3341,7 @@
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A10" s="17"/>
+      <c r="A10" s="16"/>
       <c r="B10" s="5">
         <v>3.5</v>
       </c>
@@ -3365,7 +3373,7 @@
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A11" s="17"/>
+      <c r="A11" s="16"/>
       <c r="B11" s="5">
         <v>4</v>
       </c>
@@ -3397,7 +3405,7 @@
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A12" s="17"/>
+      <c r="A12" s="16"/>
       <c r="B12" s="5">
         <v>4.5</v>
       </c>
@@ -3429,7 +3437,7 @@
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A13" s="17"/>
+      <c r="A13" s="16"/>
       <c r="B13" s="5">
         <v>5</v>
       </c>
@@ -3465,14 +3473,14 @@
       <c r="B15" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="C15" s="16" t="s">
-        <v>1</v>
-      </c>
-      <c r="D15" s="16"/>
-      <c r="E15" s="16"/>
-      <c r="F15" s="16"/>
-      <c r="G15" s="16"/>
-      <c r="H15" s="16"/>
+      <c r="C15" s="17" t="s">
+        <v>1</v>
+      </c>
+      <c r="D15" s="17"/>
+      <c r="E15" s="17"/>
+      <c r="F15" s="17"/>
+      <c r="G15" s="17"/>
+      <c r="H15" s="17"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A16" s="3"/>
@@ -3505,7 +3513,7 @@
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A17" s="17" t="s">
+      <c r="A17" s="16" t="s">
         <v>6</v>
       </c>
       <c r="B17" s="5">
@@ -3539,7 +3547,7 @@
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A18" s="17"/>
+      <c r="A18" s="16"/>
       <c r="B18" s="5">
         <v>1</v>
       </c>
@@ -3571,7 +3579,7 @@
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A19" s="17"/>
+      <c r="A19" s="16"/>
       <c r="B19" s="5">
         <v>1.5</v>
       </c>
@@ -3603,7 +3611,7 @@
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A20" s="17"/>
+      <c r="A20" s="16"/>
       <c r="B20" s="5">
         <v>2</v>
       </c>
@@ -3635,7 +3643,7 @@
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A21" s="17"/>
+      <c r="A21" s="16"/>
       <c r="B21" s="5">
         <v>2.5</v>
       </c>
@@ -3667,7 +3675,7 @@
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A22" s="17"/>
+      <c r="A22" s="16"/>
       <c r="B22" s="5">
         <v>3</v>
       </c>
@@ -3699,7 +3707,7 @@
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A23" s="17"/>
+      <c r="A23" s="16"/>
       <c r="B23" s="5">
         <v>3.5</v>
       </c>
@@ -3731,7 +3739,7 @@
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A24" s="17"/>
+      <c r="A24" s="16"/>
       <c r="B24" s="5">
         <v>4</v>
       </c>
@@ -3763,7 +3771,7 @@
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A25" s="17"/>
+      <c r="A25" s="16"/>
       <c r="B25" s="5">
         <v>4.5</v>
       </c>
@@ -3795,7 +3803,7 @@
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A26" s="17"/>
+      <c r="A26" s="16"/>
       <c r="B26" s="5">
         <v>5</v>
       </c>
@@ -3831,14 +3839,14 @@
       <c r="B28" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="C28" s="16" t="s">
+      <c r="C28" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="D28" s="16"/>
-      <c r="E28" s="16"/>
-      <c r="F28" s="16"/>
-      <c r="G28" s="16"/>
-      <c r="H28" s="16"/>
+      <c r="D28" s="17"/>
+      <c r="E28" s="17"/>
+      <c r="F28" s="17"/>
+      <c r="G28" s="17"/>
+      <c r="H28" s="17"/>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A29" s="3"/>
@@ -3871,7 +3879,7 @@
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A30" s="17" t="s">
+      <c r="A30" s="16" t="s">
         <v>6</v>
       </c>
       <c r="B30" s="5">
@@ -3905,7 +3913,7 @@
       </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A31" s="17"/>
+      <c r="A31" s="16"/>
       <c r="B31" s="5">
         <v>1</v>
       </c>
@@ -3937,7 +3945,7 @@
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A32" s="17"/>
+      <c r="A32" s="16"/>
       <c r="B32" s="5">
         <v>1.5</v>
       </c>
@@ -3969,7 +3977,7 @@
       </c>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A33" s="17"/>
+      <c r="A33" s="16"/>
       <c r="B33" s="5">
         <v>2</v>
       </c>
@@ -4001,7 +4009,7 @@
       </c>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A34" s="17"/>
+      <c r="A34" s="16"/>
       <c r="B34" s="5">
         <v>2.5</v>
       </c>
@@ -4033,7 +4041,7 @@
       </c>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A35" s="17"/>
+      <c r="A35" s="16"/>
       <c r="B35" s="5">
         <v>3</v>
       </c>
@@ -4065,7 +4073,7 @@
       </c>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A36" s="17"/>
+      <c r="A36" s="16"/>
       <c r="B36" s="5">
         <v>3.5</v>
       </c>
@@ -4097,7 +4105,7 @@
       </c>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A37" s="17"/>
+      <c r="A37" s="16"/>
       <c r="B37" s="5">
         <v>4</v>
       </c>
@@ -4129,7 +4137,7 @@
       </c>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A38" s="17"/>
+      <c r="A38" s="16"/>
       <c r="B38" s="5">
         <v>4.5</v>
       </c>
@@ -4161,7 +4169,7 @@
       </c>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A39" s="17"/>
+      <c r="A39" s="16"/>
       <c r="B39" s="5">
         <v>5</v>
       </c>
@@ -4197,14 +4205,14 @@
       <c r="B41" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="C41" s="16" t="s">
+      <c r="C41" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="D41" s="16"/>
-      <c r="E41" s="16"/>
-      <c r="F41" s="16"/>
-      <c r="G41" s="16"/>
-      <c r="H41" s="16"/>
+      <c r="D41" s="17"/>
+      <c r="E41" s="17"/>
+      <c r="F41" s="17"/>
+      <c r="G41" s="17"/>
+      <c r="H41" s="17"/>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A42" s="3"/>
@@ -4237,7 +4245,7 @@
       </c>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A43" s="17" t="s">
+      <c r="A43" s="16" t="s">
         <v>6</v>
       </c>
       <c r="B43" s="5">
@@ -4271,7 +4279,7 @@
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A44" s="17"/>
+      <c r="A44" s="16"/>
       <c r="B44" s="5">
         <v>1</v>
       </c>
@@ -4303,7 +4311,7 @@
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A45" s="17"/>
+      <c r="A45" s="16"/>
       <c r="B45" s="5">
         <v>1.5</v>
       </c>
@@ -4335,7 +4343,7 @@
       </c>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A46" s="17"/>
+      <c r="A46" s="16"/>
       <c r="B46" s="5">
         <v>2</v>
       </c>
@@ -4367,7 +4375,7 @@
       </c>
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A47" s="17"/>
+      <c r="A47" s="16"/>
       <c r="B47" s="5">
         <v>2.5</v>
       </c>
@@ -4399,7 +4407,7 @@
       </c>
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A48" s="17"/>
+      <c r="A48" s="16"/>
       <c r="B48" s="5">
         <v>3</v>
       </c>
@@ -4431,7 +4439,7 @@
       </c>
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A49" s="17"/>
+      <c r="A49" s="16"/>
       <c r="B49" s="5">
         <v>3.5</v>
       </c>
@@ -4463,7 +4471,7 @@
       </c>
     </row>
     <row r="50" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A50" s="17"/>
+      <c r="A50" s="16"/>
       <c r="B50" s="5">
         <v>4</v>
       </c>
@@ -4495,7 +4503,7 @@
       </c>
     </row>
     <row r="51" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A51" s="17"/>
+      <c r="A51" s="16"/>
       <c r="B51" s="5">
         <v>4.5</v>
       </c>
@@ -4527,7 +4535,7 @@
       </c>
     </row>
     <row r="52" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A52" s="17"/>
+      <c r="A52" s="16"/>
       <c r="B52" s="5">
         <v>5</v>
       </c>
@@ -4563,14 +4571,14 @@
       <c r="B54" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="C54" s="16" t="s">
+      <c r="C54" s="17" t="s">
         <v>12</v>
       </c>
-      <c r="D54" s="16"/>
-      <c r="E54" s="16"/>
-      <c r="F54" s="16"/>
-      <c r="G54" s="16"/>
-      <c r="H54" s="16"/>
+      <c r="D54" s="17"/>
+      <c r="E54" s="17"/>
+      <c r="F54" s="17"/>
+      <c r="G54" s="17"/>
+      <c r="H54" s="17"/>
     </row>
     <row r="55" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A55" s="3"/>
@@ -4603,7 +4611,7 @@
       </c>
     </row>
     <row r="56" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A56" s="17" t="s">
+      <c r="A56" s="16" t="s">
         <v>6</v>
       </c>
       <c r="B56" s="5">
@@ -4633,7 +4641,7 @@
       </c>
     </row>
     <row r="57" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A57" s="17"/>
+      <c r="A57" s="16"/>
       <c r="B57" s="5">
         <v>1</v>
       </c>
@@ -4661,7 +4669,7 @@
       </c>
     </row>
     <row r="58" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A58" s="17"/>
+      <c r="A58" s="16"/>
       <c r="B58" s="5">
         <v>1.5</v>
       </c>
@@ -4689,7 +4697,7 @@
       </c>
     </row>
     <row r="59" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A59" s="17"/>
+      <c r="A59" s="16"/>
       <c r="B59" s="5">
         <v>2</v>
       </c>
@@ -4717,7 +4725,7 @@
       </c>
     </row>
     <row r="60" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A60" s="17"/>
+      <c r="A60" s="16"/>
       <c r="B60" s="5">
         <v>2.5</v>
       </c>
@@ -4745,7 +4753,7 @@
       </c>
     </row>
     <row r="61" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A61" s="17"/>
+      <c r="A61" s="16"/>
       <c r="B61" s="5">
         <v>3</v>
       </c>
@@ -4773,7 +4781,7 @@
       </c>
     </row>
     <row r="62" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A62" s="17"/>
+      <c r="A62" s="16"/>
       <c r="B62" s="5">
         <v>3.5</v>
       </c>
@@ -4801,7 +4809,7 @@
       </c>
     </row>
     <row r="63" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A63" s="17"/>
+      <c r="A63" s="16"/>
       <c r="B63" s="5">
         <v>4</v>
       </c>
@@ -4829,7 +4837,7 @@
       </c>
     </row>
     <row r="64" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A64" s="17"/>
+      <c r="A64" s="16"/>
       <c r="B64" s="5">
         <v>4.5</v>
       </c>
@@ -4857,7 +4865,7 @@
       </c>
     </row>
     <row r="65" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A65" s="17"/>
+      <c r="A65" s="16"/>
       <c r="B65" s="5">
         <v>5</v>
       </c>
@@ -4889,14 +4897,14 @@
       <c r="B67" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="C67" s="16" t="s">
+      <c r="C67" s="17" t="s">
         <v>13</v>
       </c>
-      <c r="D67" s="16"/>
-      <c r="E67" s="16"/>
-      <c r="F67" s="16"/>
-      <c r="G67" s="16"/>
-      <c r="H67" s="16"/>
+      <c r="D67" s="17"/>
+      <c r="E67" s="17"/>
+      <c r="F67" s="17"/>
+      <c r="G67" s="17"/>
+      <c r="H67" s="17"/>
     </row>
     <row r="68" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A68" s="3"/>
@@ -4929,7 +4937,7 @@
       </c>
     </row>
     <row r="69" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A69" s="17" t="s">
+      <c r="A69" s="16" t="s">
         <v>6</v>
       </c>
       <c r="B69" s="5">
@@ -4959,7 +4967,7 @@
       </c>
     </row>
     <row r="70" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A70" s="17"/>
+      <c r="A70" s="16"/>
       <c r="B70" s="5">
         <v>1</v>
       </c>
@@ -4987,7 +4995,7 @@
       </c>
     </row>
     <row r="71" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A71" s="17"/>
+      <c r="A71" s="16"/>
       <c r="B71" s="5">
         <v>1.5</v>
       </c>
@@ -5015,7 +5023,7 @@
       </c>
     </row>
     <row r="72" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A72" s="17"/>
+      <c r="A72" s="16"/>
       <c r="B72" s="5">
         <v>2</v>
       </c>
@@ -5043,7 +5051,7 @@
       </c>
     </row>
     <row r="73" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A73" s="17"/>
+      <c r="A73" s="16"/>
       <c r="B73" s="5">
         <v>2.5</v>
       </c>
@@ -5071,7 +5079,7 @@
       </c>
     </row>
     <row r="74" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A74" s="17"/>
+      <c r="A74" s="16"/>
       <c r="B74" s="5">
         <v>3</v>
       </c>
@@ -5099,7 +5107,7 @@
       </c>
     </row>
     <row r="75" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A75" s="17"/>
+      <c r="A75" s="16"/>
       <c r="B75" s="5">
         <v>3.5</v>
       </c>
@@ -5127,7 +5135,7 @@
       </c>
     </row>
     <row r="76" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A76" s="17"/>
+      <c r="A76" s="16"/>
       <c r="B76" s="5">
         <v>4</v>
       </c>
@@ -5155,7 +5163,7 @@
       </c>
     </row>
     <row r="77" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A77" s="17"/>
+      <c r="A77" s="16"/>
       <c r="B77" s="5">
         <v>4.5</v>
       </c>
@@ -5183,7 +5191,7 @@
       </c>
     </row>
     <row r="78" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A78" s="17"/>
+      <c r="A78" s="16"/>
       <c r="B78" s="5">
         <v>5</v>
       </c>
@@ -5215,14 +5223,14 @@
       <c r="B80" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="C80" s="16" t="s">
+      <c r="C80" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="D80" s="16"/>
-      <c r="E80" s="16"/>
-      <c r="F80" s="16"/>
-      <c r="G80" s="16"/>
-      <c r="H80" s="16"/>
+      <c r="D80" s="17"/>
+      <c r="E80" s="17"/>
+      <c r="F80" s="17"/>
+      <c r="G80" s="17"/>
+      <c r="H80" s="17"/>
     </row>
     <row r="81" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A81" s="3"/>
@@ -5255,7 +5263,7 @@
       </c>
     </row>
     <row r="82" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A82" s="17" t="s">
+      <c r="A82" s="16" t="s">
         <v>6</v>
       </c>
       <c r="B82" s="5">
@@ -5285,7 +5293,7 @@
       </c>
     </row>
     <row r="83" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A83" s="17"/>
+      <c r="A83" s="16"/>
       <c r="B83" s="5">
         <v>1</v>
       </c>
@@ -5313,7 +5321,7 @@
       </c>
     </row>
     <row r="84" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A84" s="17"/>
+      <c r="A84" s="16"/>
       <c r="B84" s="5">
         <v>1.5</v>
       </c>
@@ -5341,7 +5349,7 @@
       </c>
     </row>
     <row r="85" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A85" s="17"/>
+      <c r="A85" s="16"/>
       <c r="B85" s="5">
         <v>2</v>
       </c>
@@ -5369,7 +5377,7 @@
       </c>
     </row>
     <row r="86" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A86" s="17"/>
+      <c r="A86" s="16"/>
       <c r="B86" s="5">
         <v>2.5</v>
       </c>
@@ -5397,7 +5405,7 @@
       </c>
     </row>
     <row r="87" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A87" s="17"/>
+      <c r="A87" s="16"/>
       <c r="B87" s="5">
         <v>3</v>
       </c>
@@ -5425,7 +5433,7 @@
       </c>
     </row>
     <row r="88" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A88" s="17"/>
+      <c r="A88" s="16"/>
       <c r="B88" s="5">
         <v>3.5</v>
       </c>
@@ -5453,7 +5461,7 @@
       </c>
     </row>
     <row r="89" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A89" s="17"/>
+      <c r="A89" s="16"/>
       <c r="B89" s="5">
         <v>4</v>
       </c>
@@ -5481,7 +5489,7 @@
       </c>
     </row>
     <row r="90" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A90" s="17"/>
+      <c r="A90" s="16"/>
       <c r="B90" s="5">
         <v>4.5</v>
       </c>
@@ -5509,7 +5517,7 @@
       </c>
     </row>
     <row r="91" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A91" s="17"/>
+      <c r="A91" s="16"/>
       <c r="B91" s="5">
         <v>5</v>
       </c>
@@ -5541,14 +5549,14 @@
       <c r="B93" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="C93" s="16" t="s">
+      <c r="C93" s="17" t="s">
         <v>16</v>
       </c>
-      <c r="D93" s="16"/>
-      <c r="E93" s="16"/>
-      <c r="F93" s="16"/>
-      <c r="G93" s="16"/>
-      <c r="H93" s="16"/>
+      <c r="D93" s="17"/>
+      <c r="E93" s="17"/>
+      <c r="F93" s="17"/>
+      <c r="G93" s="17"/>
+      <c r="H93" s="17"/>
     </row>
     <row r="94" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A94" s="3"/>
@@ -5581,7 +5589,7 @@
       </c>
     </row>
     <row r="95" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A95" s="17" t="s">
+      <c r="A95" s="16" t="s">
         <v>6</v>
       </c>
       <c r="B95" s="5">
@@ -5611,7 +5619,7 @@
       </c>
     </row>
     <row r="96" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A96" s="17"/>
+      <c r="A96" s="16"/>
       <c r="B96" s="5">
         <v>1</v>
       </c>
@@ -5639,7 +5647,7 @@
       </c>
     </row>
     <row r="97" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A97" s="17"/>
+      <c r="A97" s="16"/>
       <c r="B97" s="5">
         <v>1.5</v>
       </c>
@@ -5667,7 +5675,7 @@
       </c>
     </row>
     <row r="98" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A98" s="17"/>
+      <c r="A98" s="16"/>
       <c r="B98" s="5">
         <v>2</v>
       </c>
@@ -5695,7 +5703,7 @@
       </c>
     </row>
     <row r="99" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A99" s="17"/>
+      <c r="A99" s="16"/>
       <c r="B99" s="5">
         <v>2.5</v>
       </c>
@@ -5723,7 +5731,7 @@
       </c>
     </row>
     <row r="100" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A100" s="17"/>
+      <c r="A100" s="16"/>
       <c r="B100" s="5">
         <v>3</v>
       </c>
@@ -5751,7 +5759,7 @@
       </c>
     </row>
     <row r="101" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A101" s="17"/>
+      <c r="A101" s="16"/>
       <c r="B101" s="5">
         <v>3.5</v>
       </c>
@@ -5779,7 +5787,7 @@
       </c>
     </row>
     <row r="102" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A102" s="17"/>
+      <c r="A102" s="16"/>
       <c r="B102" s="5">
         <v>4</v>
       </c>
@@ -5807,7 +5815,7 @@
       </c>
     </row>
     <row r="103" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A103" s="17"/>
+      <c r="A103" s="16"/>
       <c r="B103" s="5">
         <v>4.5</v>
       </c>
@@ -5835,7 +5843,7 @@
       </c>
     </row>
     <row r="104" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A104" s="17"/>
+      <c r="A104" s="16"/>
       <c r="B104" s="5">
         <v>5</v>
       </c>
@@ -5864,14 +5872,6 @@
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="A82:A91"/>
-    <mergeCell ref="C93:H93"/>
-    <mergeCell ref="A95:A104"/>
-    <mergeCell ref="C54:H54"/>
-    <mergeCell ref="A56:A65"/>
-    <mergeCell ref="C67:H67"/>
-    <mergeCell ref="A69:A78"/>
-    <mergeCell ref="C80:H80"/>
     <mergeCell ref="C28:H28"/>
     <mergeCell ref="A30:A39"/>
     <mergeCell ref="C41:H41"/>
@@ -5881,6 +5881,14 @@
     <mergeCell ref="A4:A13"/>
     <mergeCell ref="C15:H15"/>
     <mergeCell ref="A17:A26"/>
+    <mergeCell ref="A82:A91"/>
+    <mergeCell ref="C93:H93"/>
+    <mergeCell ref="A95:A104"/>
+    <mergeCell ref="C54:H54"/>
+    <mergeCell ref="A56:A65"/>
+    <mergeCell ref="C67:H67"/>
+    <mergeCell ref="A69:A78"/>
+    <mergeCell ref="C80:H80"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -23560,4 +23568,1096 @@
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{109F14CE-F985-7647-A891-E76A90D01467}">
+  <dimension ref="A1:J71"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:10" ht="34" x14ac:dyDescent="0.2">
+      <c r="A1" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="I1" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1" s="19" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>0.5</v>
+      </c>
+      <c r="H2">
+        <f>SUM(A2:G2)</f>
+        <v>0.5</v>
+      </c>
+      <c r="I2">
+        <v>99.326800000000006</v>
+      </c>
+      <c r="J2">
+        <v>3.804248242333824</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>1</v>
+      </c>
+      <c r="H3">
+        <f t="shared" ref="H3:H66" si="0">SUM(A3:G3)</f>
+        <v>1</v>
+      </c>
+      <c r="I3">
+        <v>96.763745000000014</v>
+      </c>
+      <c r="J3">
+        <v>3.5137884775113677</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A4">
+        <v>1.5</v>
+      </c>
+      <c r="H4">
+        <f t="shared" si="0"/>
+        <v>1.5</v>
+      </c>
+      <c r="I4">
+        <v>91.502356666666671</v>
+      </c>
+      <c r="J4">
+        <v>6.7555134782799628</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A5">
+        <v>2</v>
+      </c>
+      <c r="H5">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="I5">
+        <v>85.783123333333336</v>
+      </c>
+      <c r="J5">
+        <v>3.492629492133716</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A6">
+        <v>2.5</v>
+      </c>
+      <c r="H6">
+        <f t="shared" si="0"/>
+        <v>2.5</v>
+      </c>
+      <c r="I6">
+        <v>85.148414999999986</v>
+      </c>
+      <c r="J6">
+        <v>4.2892130931393844</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A7">
+        <v>3</v>
+      </c>
+      <c r="H7">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="I7">
+        <v>83.938525000000013</v>
+      </c>
+      <c r="J7">
+        <v>6.7398799167511134</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A8">
+        <v>3.5</v>
+      </c>
+      <c r="H8">
+        <f t="shared" si="0"/>
+        <v>3.5</v>
+      </c>
+      <c r="I8">
+        <v>79.902073333333334</v>
+      </c>
+      <c r="J8">
+        <v>7.0862700694739447</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A9">
+        <v>4</v>
+      </c>
+      <c r="H9">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="I9">
+        <v>69.552929999999989</v>
+      </c>
+      <c r="J9">
+        <v>13.314279827890326</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A10">
+        <v>4.5</v>
+      </c>
+      <c r="H10">
+        <f t="shared" si="0"/>
+        <v>4.5</v>
+      </c>
+      <c r="I10">
+        <v>46.883814999999998</v>
+      </c>
+      <c r="J10">
+        <v>11.3053488463039</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A11">
+        <v>5</v>
+      </c>
+      <c r="H11">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="I11">
+        <v>25.455936666666663</v>
+      </c>
+      <c r="J11">
+        <v>8.9999707442722077</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="B12">
+        <v>0.5</v>
+      </c>
+      <c r="H12">
+        <f t="shared" si="0"/>
+        <v>0.5</v>
+      </c>
+      <c r="I12">
+        <v>93.389521666666667</v>
+      </c>
+      <c r="J12">
+        <v>3.6986545303547707</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="B13">
+        <v>1</v>
+      </c>
+      <c r="H13">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="I13">
+        <v>81.105253333333323</v>
+      </c>
+      <c r="J13">
+        <v>4.1793786424366459</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="B14">
+        <v>1.5</v>
+      </c>
+      <c r="H14">
+        <f t="shared" si="0"/>
+        <v>1.5</v>
+      </c>
+      <c r="I14">
+        <v>73.02797333333335</v>
+      </c>
+      <c r="J14">
+        <v>4.7345333865498898</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="B15">
+        <v>2</v>
+      </c>
+      <c r="H15">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="I15">
+        <v>65.395256666666654</v>
+      </c>
+      <c r="J15">
+        <v>5.7035398470706093</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="B16">
+        <v>2.5</v>
+      </c>
+      <c r="H16">
+        <f t="shared" si="0"/>
+        <v>2.5</v>
+      </c>
+      <c r="I16">
+        <v>63.903803333333322</v>
+      </c>
+      <c r="J16">
+        <v>4.4590465276509006</v>
+      </c>
+    </row>
+    <row r="17" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B17">
+        <v>3</v>
+      </c>
+      <c r="H17">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="I17">
+        <v>60.433103333333328</v>
+      </c>
+      <c r="J17">
+        <v>3.8926162528418953</v>
+      </c>
+    </row>
+    <row r="18" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B18">
+        <v>3.5</v>
+      </c>
+      <c r="H18">
+        <f t="shared" si="0"/>
+        <v>3.5</v>
+      </c>
+      <c r="I18">
+        <v>54.030618333333337</v>
+      </c>
+      <c r="J18">
+        <v>5.7367173484330731</v>
+      </c>
+    </row>
+    <row r="19" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B19">
+        <v>4</v>
+      </c>
+      <c r="H19">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="I19">
+        <v>37.36924166666666</v>
+      </c>
+      <c r="J19">
+        <v>5.9455680850821402</v>
+      </c>
+    </row>
+    <row r="20" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B20">
+        <v>4.5</v>
+      </c>
+      <c r="H20">
+        <f t="shared" si="0"/>
+        <v>4.5</v>
+      </c>
+      <c r="I20">
+        <v>29.045523333333335</v>
+      </c>
+      <c r="J20">
+        <v>4.919191770913403</v>
+      </c>
+    </row>
+    <row r="21" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B21">
+        <v>5</v>
+      </c>
+      <c r="H21">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="I21">
+        <v>16.665073333333336</v>
+      </c>
+      <c r="J21">
+        <v>6.6065807453292731</v>
+      </c>
+    </row>
+    <row r="22" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="C22">
+        <v>0.5</v>
+      </c>
+      <c r="H22">
+        <f t="shared" si="0"/>
+        <v>0.5</v>
+      </c>
+      <c r="I22">
+        <v>100.65658833333333</v>
+      </c>
+      <c r="J22">
+        <v>4.8186854880814991</v>
+      </c>
+    </row>
+    <row r="23" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="C23">
+        <v>1</v>
+      </c>
+      <c r="H23">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="I23">
+        <v>103.59732666666667</v>
+      </c>
+      <c r="J23">
+        <v>6.3563255282164031</v>
+      </c>
+    </row>
+    <row r="24" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="C24">
+        <v>1.5</v>
+      </c>
+      <c r="H24">
+        <f t="shared" si="0"/>
+        <v>1.5</v>
+      </c>
+      <c r="I24">
+        <v>96.026041666666671</v>
+      </c>
+      <c r="J24">
+        <v>5.763821127826624</v>
+      </c>
+    </row>
+    <row r="25" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="C25">
+        <v>2</v>
+      </c>
+      <c r="H25">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="I25">
+        <v>95.932315000000003</v>
+      </c>
+      <c r="J25">
+        <v>5.3446851811799911</v>
+      </c>
+    </row>
+    <row r="26" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="C26">
+        <v>2.5</v>
+      </c>
+      <c r="H26">
+        <f t="shared" si="0"/>
+        <v>2.5</v>
+      </c>
+      <c r="I26">
+        <v>94.762564999999995</v>
+      </c>
+      <c r="J26">
+        <v>7.3512749100246797</v>
+      </c>
+    </row>
+    <row r="27" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="C27">
+        <v>3</v>
+      </c>
+      <c r="H27">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="I27">
+        <v>96.561785</v>
+      </c>
+      <c r="J27">
+        <v>7.9839963770298024</v>
+      </c>
+    </row>
+    <row r="28" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="C28">
+        <v>3.5</v>
+      </c>
+      <c r="H28">
+        <f t="shared" si="0"/>
+        <v>3.5</v>
+      </c>
+      <c r="I28">
+        <v>93.562100000000001</v>
+      </c>
+      <c r="J28">
+        <v>8.0542113619832456</v>
+      </c>
+    </row>
+    <row r="29" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="C29">
+        <v>4</v>
+      </c>
+      <c r="H29">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="I29">
+        <v>90.170388333333335</v>
+      </c>
+      <c r="J29">
+        <v>3.7120306348296621</v>
+      </c>
+    </row>
+    <row r="30" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="C30">
+        <v>4.5</v>
+      </c>
+      <c r="H30">
+        <f t="shared" si="0"/>
+        <v>4.5</v>
+      </c>
+      <c r="I30">
+        <v>87.89191666666666</v>
+      </c>
+      <c r="J30">
+        <v>5.439480570454827</v>
+      </c>
+    </row>
+    <row r="31" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="C31">
+        <v>5</v>
+      </c>
+      <c r="H31">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="I31">
+        <v>83.256373333333329</v>
+      </c>
+      <c r="J31">
+        <v>5.3649680301118519</v>
+      </c>
+    </row>
+    <row r="32" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="D32">
+        <v>0.5</v>
+      </c>
+      <c r="H32">
+        <f t="shared" si="0"/>
+        <v>0.5</v>
+      </c>
+      <c r="I32">
+        <v>100.26775666666667</v>
+      </c>
+      <c r="J32">
+        <v>4.8461671132647597</v>
+      </c>
+    </row>
+    <row r="33" spans="4:10" x14ac:dyDescent="0.2">
+      <c r="D33">
+        <v>1</v>
+      </c>
+      <c r="H33">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="I33">
+        <v>92.040413333333333</v>
+      </c>
+      <c r="J33">
+        <v>2.7357367186961219</v>
+      </c>
+    </row>
+    <row r="34" spans="4:10" x14ac:dyDescent="0.2">
+      <c r="D34">
+        <v>1.5</v>
+      </c>
+      <c r="H34">
+        <f t="shared" si="0"/>
+        <v>1.5</v>
+      </c>
+      <c r="I34">
+        <v>91.675261666666657</v>
+      </c>
+      <c r="J34">
+        <v>3.9410983952337322</v>
+      </c>
+    </row>
+    <row r="35" spans="4:10" x14ac:dyDescent="0.2">
+      <c r="D35">
+        <v>2</v>
+      </c>
+      <c r="H35">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="I35">
+        <v>91.344608333333326</v>
+      </c>
+      <c r="J35">
+        <v>3.4326496866289564</v>
+      </c>
+    </row>
+    <row r="36" spans="4:10" x14ac:dyDescent="0.2">
+      <c r="D36">
+        <v>2.5</v>
+      </c>
+      <c r="H36">
+        <f t="shared" si="0"/>
+        <v>2.5</v>
+      </c>
+      <c r="I36">
+        <v>91.950903333333329</v>
+      </c>
+      <c r="J36">
+        <v>3.8914788347947566</v>
+      </c>
+    </row>
+    <row r="37" spans="4:10" x14ac:dyDescent="0.2">
+      <c r="D37">
+        <v>3</v>
+      </c>
+      <c r="H37">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="I37">
+        <v>88.205523333333346</v>
+      </c>
+      <c r="J37">
+        <v>7.0424800561891683</v>
+      </c>
+    </row>
+    <row r="38" spans="4:10" x14ac:dyDescent="0.2">
+      <c r="D38">
+        <v>3.5</v>
+      </c>
+      <c r="H38">
+        <f t="shared" si="0"/>
+        <v>3.5</v>
+      </c>
+      <c r="I38">
+        <v>82.51456499999999</v>
+      </c>
+      <c r="J38">
+        <v>7.1439783297444501</v>
+      </c>
+    </row>
+    <row r="39" spans="4:10" x14ac:dyDescent="0.2">
+      <c r="D39">
+        <v>4</v>
+      </c>
+      <c r="H39">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="I39">
+        <v>64.748963333333322</v>
+      </c>
+      <c r="J39">
+        <v>9.3295049106311261</v>
+      </c>
+    </row>
+    <row r="40" spans="4:10" x14ac:dyDescent="0.2">
+      <c r="D40">
+        <v>4.5</v>
+      </c>
+      <c r="H40">
+        <f t="shared" si="0"/>
+        <v>4.5</v>
+      </c>
+      <c r="I40">
+        <v>13.690333666666668</v>
+      </c>
+      <c r="J40">
+        <v>10.211145487994521</v>
+      </c>
+    </row>
+    <row r="41" spans="4:10" x14ac:dyDescent="0.2">
+      <c r="D41">
+        <v>5</v>
+      </c>
+      <c r="H41">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="I41">
+        <v>3.4673855000000002</v>
+      </c>
+      <c r="J41">
+        <v>5.4982170691889678</v>
+      </c>
+    </row>
+    <row r="42" spans="4:10" x14ac:dyDescent="0.2">
+      <c r="E42">
+        <v>0.5</v>
+      </c>
+      <c r="H42">
+        <f t="shared" si="0"/>
+        <v>0.5</v>
+      </c>
+      <c r="I42">
+        <v>96.990867499999993</v>
+      </c>
+      <c r="J42">
+        <v>3.5244283899547093</v>
+      </c>
+    </row>
+    <row r="43" spans="4:10" x14ac:dyDescent="0.2">
+      <c r="E43">
+        <v>1</v>
+      </c>
+      <c r="H43">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="I43">
+        <v>88.637667500000006</v>
+      </c>
+      <c r="J43">
+        <v>3.446098477803381</v>
+      </c>
+    </row>
+    <row r="44" spans="4:10" x14ac:dyDescent="0.2">
+      <c r="E44">
+        <v>1.5</v>
+      </c>
+      <c r="H44">
+        <f t="shared" si="0"/>
+        <v>1.5</v>
+      </c>
+      <c r="I44">
+        <v>86.018712499999992</v>
+      </c>
+      <c r="J44">
+        <v>4.2165751997466785</v>
+      </c>
+    </row>
+    <row r="45" spans="4:10" x14ac:dyDescent="0.2">
+      <c r="E45">
+        <v>2</v>
+      </c>
+      <c r="H45">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="I45">
+        <v>80.965107500000002</v>
+      </c>
+      <c r="J45">
+        <v>4.8955379709301372</v>
+      </c>
+    </row>
+    <row r="46" spans="4:10" x14ac:dyDescent="0.2">
+      <c r="E46">
+        <v>2.5</v>
+      </c>
+      <c r="H46">
+        <f t="shared" si="0"/>
+        <v>2.5</v>
+      </c>
+      <c r="I46">
+        <v>77.546895000000006</v>
+      </c>
+      <c r="J46">
+        <v>1.8660118111295516</v>
+      </c>
+    </row>
+    <row r="47" spans="4:10" x14ac:dyDescent="0.2">
+      <c r="E47">
+        <v>3</v>
+      </c>
+      <c r="H47">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="I47">
+        <v>75.391487499999997</v>
+      </c>
+      <c r="J47">
+        <v>2.5370125913007917</v>
+      </c>
+    </row>
+    <row r="48" spans="4:10" x14ac:dyDescent="0.2">
+      <c r="E48">
+        <v>3.5</v>
+      </c>
+      <c r="H48">
+        <f t="shared" si="0"/>
+        <v>3.5</v>
+      </c>
+      <c r="I48">
+        <v>67.414590000000004</v>
+      </c>
+      <c r="J48">
+        <v>4.5515080294722114</v>
+      </c>
+    </row>
+    <row r="49" spans="5:10" x14ac:dyDescent="0.2">
+      <c r="E49">
+        <v>4</v>
+      </c>
+      <c r="H49">
+        <f>SUM(A49:G49)</f>
+        <v>4</v>
+      </c>
+      <c r="I49">
+        <v>58.287497499999994</v>
+      </c>
+      <c r="J49">
+        <v>3.7058015183720721</v>
+      </c>
+    </row>
+    <row r="50" spans="5:10" x14ac:dyDescent="0.2">
+      <c r="E50">
+        <v>4.5</v>
+      </c>
+      <c r="H50">
+        <f t="shared" si="0"/>
+        <v>4.5</v>
+      </c>
+      <c r="I50">
+        <v>54.744797500000004</v>
+      </c>
+      <c r="J50">
+        <v>3.2831516321925722</v>
+      </c>
+    </row>
+    <row r="51" spans="5:10" x14ac:dyDescent="0.2">
+      <c r="E51">
+        <v>5</v>
+      </c>
+      <c r="H51">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="I51">
+        <v>48.984327500000006</v>
+      </c>
+      <c r="J51">
+        <v>2.3987734419320952</v>
+      </c>
+    </row>
+    <row r="52" spans="5:10" x14ac:dyDescent="0.2">
+      <c r="F52">
+        <v>0.5</v>
+      </c>
+      <c r="H52">
+        <f t="shared" si="0"/>
+        <v>0.5</v>
+      </c>
+      <c r="I52">
+        <v>103.63339999999999</v>
+      </c>
+      <c r="J52">
+        <v>5.5578065578967371</v>
+      </c>
+    </row>
+    <row r="53" spans="5:10" x14ac:dyDescent="0.2">
+      <c r="F53">
+        <v>1</v>
+      </c>
+      <c r="H53">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="I53">
+        <v>92.954874999999987</v>
+      </c>
+      <c r="J53">
+        <v>4.0768949617846424</v>
+      </c>
+    </row>
+    <row r="54" spans="5:10" x14ac:dyDescent="0.2">
+      <c r="F54">
+        <v>1.5</v>
+      </c>
+      <c r="H54">
+        <f t="shared" si="0"/>
+        <v>1.5</v>
+      </c>
+      <c r="I54">
+        <v>89.473919999999993</v>
+      </c>
+      <c r="J54">
+        <v>0.87185287256509103</v>
+      </c>
+    </row>
+    <row r="55" spans="5:10" x14ac:dyDescent="0.2">
+      <c r="F55">
+        <v>2</v>
+      </c>
+      <c r="H55">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="I55">
+        <v>85.191647500000002</v>
+      </c>
+      <c r="J55">
+        <v>2.625736718117174</v>
+      </c>
+    </row>
+    <row r="56" spans="5:10" x14ac:dyDescent="0.2">
+      <c r="F56">
+        <v>2.5</v>
+      </c>
+      <c r="H56">
+        <f t="shared" si="0"/>
+        <v>2.5</v>
+      </c>
+      <c r="I56">
+        <v>85.460427500000009</v>
+      </c>
+      <c r="J56">
+        <v>1.7168374177157126</v>
+      </c>
+    </row>
+    <row r="57" spans="5:10" x14ac:dyDescent="0.2">
+      <c r="F57">
+        <v>3</v>
+      </c>
+      <c r="H57">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="I57">
+        <v>75.961699999999993</v>
+      </c>
+      <c r="J57">
+        <v>2.6418689499386598</v>
+      </c>
+    </row>
+    <row r="58" spans="5:10" x14ac:dyDescent="0.2">
+      <c r="F58">
+        <v>3.5</v>
+      </c>
+      <c r="H58">
+        <f t="shared" si="0"/>
+        <v>3.5</v>
+      </c>
+      <c r="I58">
+        <v>71.401984999999996</v>
+      </c>
+      <c r="J58">
+        <v>5.6160800933502575</v>
+      </c>
+    </row>
+    <row r="59" spans="5:10" x14ac:dyDescent="0.2">
+      <c r="F59">
+        <v>4</v>
+      </c>
+      <c r="H59">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="I59">
+        <v>60.172202500000004</v>
+      </c>
+      <c r="J59">
+        <v>7.0975126007333253</v>
+      </c>
+    </row>
+    <row r="60" spans="5:10" x14ac:dyDescent="0.2">
+      <c r="F60">
+        <v>4.5</v>
+      </c>
+      <c r="H60">
+        <f t="shared" si="0"/>
+        <v>4.5</v>
+      </c>
+      <c r="I60">
+        <v>39.883452500000004</v>
+      </c>
+      <c r="J60">
+        <v>9.9313472568916197</v>
+      </c>
+    </row>
+    <row r="61" spans="5:10" x14ac:dyDescent="0.2">
+      <c r="F61">
+        <v>5</v>
+      </c>
+      <c r="H61">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="I61">
+        <v>16.1445075</v>
+      </c>
+      <c r="J61">
+        <v>1.9281371330039641</v>
+      </c>
+    </row>
+    <row r="62" spans="5:10" x14ac:dyDescent="0.2">
+      <c r="G62">
+        <v>0.5</v>
+      </c>
+      <c r="H62">
+        <f t="shared" si="0"/>
+        <v>0.5</v>
+      </c>
+      <c r="I62">
+        <v>80.549022499999992</v>
+      </c>
+      <c r="J62">
+        <v>5.0579088447666507</v>
+      </c>
+    </row>
+    <row r="63" spans="5:10" x14ac:dyDescent="0.2">
+      <c r="G63">
+        <v>1</v>
+      </c>
+      <c r="H63">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="I63">
+        <v>78.555360000000007</v>
+      </c>
+      <c r="J63">
+        <v>8.5711359912557477</v>
+      </c>
+    </row>
+    <row r="64" spans="5:10" x14ac:dyDescent="0.2">
+      <c r="G64">
+        <v>1.5</v>
+      </c>
+      <c r="H64">
+        <f t="shared" si="0"/>
+        <v>1.5</v>
+      </c>
+      <c r="I64">
+        <v>46.349990000000005</v>
+      </c>
+      <c r="J64">
+        <v>2.8540384281663043</v>
+      </c>
+    </row>
+    <row r="65" spans="7:10" x14ac:dyDescent="0.2">
+      <c r="G65">
+        <v>2</v>
+      </c>
+      <c r="H65">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="I65">
+        <v>28.72598</v>
+      </c>
+      <c r="J65">
+        <v>4.4012179564581837</v>
+      </c>
+    </row>
+    <row r="66" spans="7:10" x14ac:dyDescent="0.2">
+      <c r="G66">
+        <v>2.5</v>
+      </c>
+      <c r="H66">
+        <f t="shared" si="0"/>
+        <v>2.5</v>
+      </c>
+      <c r="I66">
+        <v>16.474955000000001</v>
+      </c>
+      <c r="J66">
+        <v>3.7628059888233585</v>
+      </c>
+    </row>
+    <row r="67" spans="7:10" x14ac:dyDescent="0.2">
+      <c r="G67">
+        <v>3</v>
+      </c>
+      <c r="H67">
+        <f t="shared" ref="H67:H71" si="1">SUM(A67:G67)</f>
+        <v>3</v>
+      </c>
+      <c r="I67">
+        <v>6.2579514999999999</v>
+      </c>
+      <c r="J67">
+        <v>1.3039370241097741</v>
+      </c>
+    </row>
+    <row r="68" spans="7:10" x14ac:dyDescent="0.2">
+      <c r="G68">
+        <v>3.5</v>
+      </c>
+      <c r="H68">
+        <f t="shared" si="1"/>
+        <v>3.5</v>
+      </c>
+      <c r="I68">
+        <v>0.26893024999999998</v>
+      </c>
+      <c r="J68">
+        <v>8.5463924688651466E-2</v>
+      </c>
+    </row>
+    <row r="69" spans="7:10" x14ac:dyDescent="0.2">
+      <c r="G69">
+        <v>4</v>
+      </c>
+      <c r="H69">
+        <f t="shared" si="1"/>
+        <v>4</v>
+      </c>
+      <c r="I69">
+        <v>-6.0808500000000001E-2</v>
+      </c>
+      <c r="J69">
+        <v>0.10613757090093026</v>
+      </c>
+    </row>
+    <row r="70" spans="7:10" x14ac:dyDescent="0.2">
+      <c r="G70">
+        <v>4.5</v>
+      </c>
+      <c r="H70">
+        <f t="shared" si="1"/>
+        <v>4.5</v>
+      </c>
+      <c r="I70">
+        <v>-6.0029249999999992E-2</v>
+      </c>
+      <c r="J70">
+        <v>0.10581291769763983</v>
+      </c>
+    </row>
+    <row r="71" spans="7:10" x14ac:dyDescent="0.2">
+      <c r="G71">
+        <v>5</v>
+      </c>
+      <c r="H71">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="I71">
+        <v>-0.13352250000000002</v>
+      </c>
+      <c r="J71">
+        <v>4.2628885966560247E-2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>